<commit_message>
Prompt coach live test: plant known answers in FR-1, FR-3, FR-4
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sp6bbiPXfwDc65dz8hiGei
</commit_message>
<xml_diff>
--- a/prompt-coach/research/live-tests/fixtures/fr_accruals.xlsx
+++ b/prompt-coach/research/live-tests/fixtures/fr_accruals.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,9 +483,23 @@
         <v>Q3 bonus</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>JE-106</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Accrued freight</v>
+      </c>
+      <c r="C7">
+        <v>12</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Sept freight</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>